<commit_message>
finished ui, added dynamic resize for alle except flashing bade pitmode. not just need to test with uart signal
</commit_message>
<xml_diff>
--- a/dashboard/object_id.xlsx
+++ b/dashboard/object_id.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet name="Page 1 UI Elements" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Page 2 UI Elements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Python Dicts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Page 10 UI Elements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Python Dicts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -997,7 +998,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>2</t>
@@ -1025,7 +1025,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>2</t>
@@ -1053,7 +1052,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>2</t>
@@ -1081,7 +1079,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>2</t>
@@ -1099,12 +1096,533 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A71"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>class_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>default_value</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tireFLValue</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tireFRValue</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tireRLValue</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tireRRValue</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>maxCellValue</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>maxCellBar</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>speedValue</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>km/h</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>psiFLValue</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PSI</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>psiFRValue</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PSI</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>28</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>psiRLValue</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PSI</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>29</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>psiRRValue</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PSI</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>30</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>socValue</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>31</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>socBar</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>32</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>brakeBar</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>33</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>throttleBar</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>34</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cardPitMode</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>badge</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t># id dictionary</t>
         </is>
       </c>
@@ -1252,336 +1770,700 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+          <t xml:space="preserve">    # page_10</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    19: "tireFLValue",</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t># uart_data dictionary</t>
+          <t xml:space="preserve">    20: "tireFRValue",</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>uart_data = {</t>
+          <t xml:space="preserve">    21: "tireRLValue",</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "frontbrakebar": 0,</t>
+          <t xml:space="preserve">    22: "tireRRValue",</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "rearbrakebar": 0,</t>
+          <t xml:space="preserve">    23: "maxCellValue",</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "speedbar": 0,</t>
+          <t xml:space="preserve">    24: "maxCellBar",</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "throttlebar": 0,</t>
+          <t xml:space="preserve">    25: "speedValue",</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "front_brake_text": 0,</t>
+          <t xml:space="preserve">    26: "psiFLValue",</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "rear_brake_text": 0,</t>
+          <t xml:space="preserve">    27: "psiFRValue",</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "speed_text": 0,</t>
+          <t xml:space="preserve">    28: "psiRLValue",</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "throttle_text": 0,</t>
+          <t xml:space="preserve">    29: "psiRRValue",</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # page_2</t>
+          <t xml:space="preserve">    30: "socValue",</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "valCurrent": 0,</t>
+          <t xml:space="preserve">    31: "socBar",</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "valVoltage": 0,</t>
+          <t xml:space="preserve">    32: "brakeBar",</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "valMinTemp": 0,</t>
+          <t xml:space="preserve">    33: "throttleBar",</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "valMaxTemp": 0,</t>
+          <t xml:space="preserve">    34: "cardPitMode",</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "valMinVolt": 0,</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    "valMaxVolt": 0,</t>
-        </is>
-      </c>
-    </row>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "badgeCharging": 0,</t>
+          <t># uart_data dictionary</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "badgeBalancing": 0,</t>
+          <t>uart_data = {</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "dotCharging": 0,</t>
+          <t xml:space="preserve">    "frontbrakebar": 0,</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "dotBalancing": 0,</t>
+          <t xml:space="preserve">    "rearbrakebar": 0,</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>}</t>
-        </is>
-      </c>
-    </row>
-    <row r="46"/>
+          <t xml:space="preserve">    "speedbar": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "throttlebar": 0,</t>
+        </is>
+      </c>
+    </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t># pages dictionary</t>
+          <t xml:space="preserve">    "front_brake_text": 0,</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>pages = {</t>
+          <t xml:space="preserve">    "rear_brake_text": 0,</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "page_1": {</t>
+          <t xml:space="preserve">    "speed_text": 0,</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "frontbrakebar": "bar",</t>
+          <t xml:space="preserve">    "throttle_text": 0,</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rearbrakebar": "bar",</t>
+          <t xml:space="preserve">    # page_2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "speedbar": "bar",</t>
+          <t xml:space="preserve">    "valCurrent": 0,</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "throttlebar": "bar",</t>
+          <t xml:space="preserve">    "valVoltage": 0,</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "front_brake_text": "text",</t>
+          <t xml:space="preserve">    "valMinTemp": 0,</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rear_brake_text": "text",</t>
+          <t xml:space="preserve">    "valMaxTemp": 0,</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "speed_text": "text",</t>
+          <t xml:space="preserve">    "valMinVolt": 0,</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "throttle_text": "text",</t>
+          <t xml:space="preserve">    "valMaxVolt": 0,</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    },</t>
+          <t xml:space="preserve">    "badgeCharging": 0,</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "page_2": {</t>
+          <t xml:space="preserve">    "badgeBalancing": 0,</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "valCurrent": "text",</t>
+          <t xml:space="preserve">    "dotCharging": 0,</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "valVoltage": "text",</t>
+          <t xml:space="preserve">    "dotBalancing": 0,</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "valMinTemp": "text",</t>
+          <t xml:space="preserve">    # page_10</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "valMaxTemp": "text",</t>
+          <t xml:space="preserve">    "tireFLValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "valMinVolt": "text",</t>
+          <t xml:space="preserve">    "tireFRValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "valMaxVolt": "text",</t>
+          <t xml:space="preserve">    "tireRLValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "badgeCharging": "badge",</t>
+          <t xml:space="preserve">    "tireRRValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "badgeBalancing": "badge",</t>
+          <t xml:space="preserve">    "maxCellValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "dotCharging": "led",</t>
+          <t xml:space="preserve">    "maxCellBar": 0,</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "dotBalancing": "led",</t>
+          <t xml:space="preserve">    "speedValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">    },</t>
+          <t xml:space="preserve">    "psiFLValue": 0,</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "psiFRValue": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "psiRLValue": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "psiRRValue": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "socValue": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "socBar": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "brakeBar": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "throttleBar": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "cardPitMode": 0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="80"/>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t># pages dictionary</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>pages = {</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "page_1": {</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "frontbrakebar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "rearbrakebar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "speedbar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "throttlebar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "front_brake_text": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "rear_brake_text": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "speed_text": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "throttle_text": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    },</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "page_2": {</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "valCurrent": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "valVoltage": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "valMinTemp": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "valMaxTemp": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "valMinVolt": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "valMaxVolt": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "badgeCharging": "badge",</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "badgeBalancing": "badge",</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "dotCharging": "led",</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "dotBalancing": "led",</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    },</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "page_10": {</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "tireFLValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "tireFRValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "tireRLValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "tireRRValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "maxCellValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "maxCellBar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "speedValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "psiFLValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "psiFRValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "psiRLValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "psiRRValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "socValue": "text",</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "socBar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "brakeBar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "throttleBar": "bar",</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "cardPitMode": "badge",</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    },</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
         <is>
           <t>}</t>
         </is>

</xml_diff>